<commit_message>
new workload component and optimization model
</commit_message>
<xml_diff>
--- a/dataset/Data_annex_Energy_and_AI.xlsx
+++ b/dataset/Data_annex_Energy_and_AI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\我的云端硬盘\☆_論文\sci\22_NatureSustainability\dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AIfootprint\Code\dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06A4CD9C-3B38-4707-9DCF-39A640DA2F91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A2B00D1-4A65-43B6-A168-394F0CC764F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{D7B4F2E1-D24B-4A1B-B9F3-C15A28CCB8C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="32640" windowHeight="21120" activeTab="1" xr2:uid="{D7B4F2E1-D24B-4A1B-B9F3-C15A28CCB8C7}"/>
   </bookViews>
   <sheets>
     <sheet name="World Data" sheetId="1" r:id="rId1"/>
@@ -235,7 +235,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="13">
+  <numFmts count="15">
     <numFmt numFmtId="176" formatCode="#\ ##0\ \ \ \ ;\-#\ ##0\ \ \ \ ;\-\ \ \ \ "/>
     <numFmt numFmtId="177" formatCode="#\ ##0\ \ ;\-#\ ##0\ \ ;\-\ \ "/>
     <numFmt numFmtId="178" formatCode="0\ ;\-0\ ;\-\ "/>
@@ -249,6 +249,8 @@
     <numFmt numFmtId="186" formatCode="##.00\ \ ;\-##.00\ \ ;\-\ \ "/>
     <numFmt numFmtId="187" formatCode="0\ "/>
     <numFmt numFmtId="188" formatCode="#.0\ ##0\ \ \ \ ;\-#.0\ ##0\ \ \ \ ;\-\ \ \ \ "/>
+    <numFmt numFmtId="193" formatCode="0.0_);[Red]\(0.0\)"/>
+    <numFmt numFmtId="194" formatCode="0.00_);[Red]\(0.00\)"/>
   </numFmts>
   <fonts count="16" x14ac:knownFonts="1">
     <font>
@@ -527,7 +529,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -835,6 +837,8 @@
     <xf numFmtId="182" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="193" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="194" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -857,6 +861,1050 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="zh-CN"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Regional Data'!$B$66</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>IT electricity consumption (TWh)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Regional Data'!$C$55:$G$55</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2030</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Regional Data'!$C$67:$G$67</c:f>
+              <c:numCache>
+                <c:formatCode>#\ ##0\ \ \ \ ;\-#\ ##0\ \ \ \ ;\-\ \ \ \ </c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>176</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>252</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>295</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="0\ ;\-0\ ;\-\ ">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>733</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-350C-47B3-831E-E8DC31DE67CF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Regional Data'!$B$56</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total electricity consumption (TWh)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Regional Data'!$C$55:$G$55</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>2020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2030</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Regional Data'!$C$57:$G$57</c:f>
+              <c:numCache>
+                <c:formatCode>#\ ##0\ \ \ \ ;\-#\ ##0\ \ \ \ ;\-\ \ \ \ </c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>269</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>361</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>416</c:v>
+                </c:pt>
+                <c:pt idx="3" formatCode="0\ ;\-0\ ;\-\ ">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>946</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-350C-47B3-831E-E8DC31DE67CF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="2003820623"/>
+        <c:axId val="1974361935"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="2003820623"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1974361935"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1974361935"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#\ ##0\ \ \ \ ;\-#\ ##0\ \ \ \ ;\-\ \ \ \ " sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2003820623"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>414008</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>150100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>571171</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>37606</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="图表 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{50B7FDD5-F4A4-7863-FC7E-4912C0EA68B3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1178,33 +2226,33 @@
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:AI37"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="2" max="2" width="0.453125" customWidth="1"/>
-    <col min="3" max="3" width="24.1796875" customWidth="1"/>
-    <col min="4" max="6" width="5.7265625" customWidth="1"/>
-    <col min="7" max="7" width="0.1796875" style="18" customWidth="1"/>
-    <col min="8" max="8" width="5.7265625" style="83" customWidth="1"/>
-    <col min="9" max="9" width="5.7265625" customWidth="1"/>
-    <col min="10" max="10" width="0.54296875" style="18" customWidth="1"/>
-    <col min="11" max="11" width="5.7265625" style="83" customWidth="1"/>
-    <col min="12" max="12" width="5.7265625" customWidth="1"/>
-    <col min="13" max="13" width="0.54296875" style="18" customWidth="1"/>
-    <col min="14" max="14" width="5.7265625" style="83" customWidth="1"/>
-    <col min="15" max="15" width="5.7265625" customWidth="1"/>
-    <col min="16" max="16" width="0.54296875" style="18" customWidth="1"/>
-    <col min="17" max="18" width="5.7265625" customWidth="1"/>
-    <col min="19" max="19" width="0.26953125" style="18" customWidth="1"/>
+    <col min="2" max="2" width="0.5" customWidth="1"/>
+    <col min="3" max="3" width="24.125" customWidth="1"/>
+    <col min="4" max="6" width="5.75" customWidth="1"/>
+    <col min="7" max="7" width="0.125" style="18" customWidth="1"/>
+    <col min="8" max="8" width="5.75" style="83" customWidth="1"/>
+    <col min="9" max="9" width="5.75" customWidth="1"/>
+    <col min="10" max="10" width="0.5" style="18" customWidth="1"/>
+    <col min="11" max="11" width="5.75" style="83" customWidth="1"/>
+    <col min="12" max="12" width="5.75" customWidth="1"/>
+    <col min="13" max="13" width="0.5" style="18" customWidth="1"/>
+    <col min="14" max="14" width="5.75" style="83" customWidth="1"/>
+    <col min="15" max="15" width="5.75" customWidth="1"/>
+    <col min="16" max="16" width="0.5" style="18" customWidth="1"/>
+    <col min="17" max="18" width="5.75" customWidth="1"/>
+    <col min="19" max="19" width="0.25" style="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.15">
       <c r="G1" s="11"/>
       <c r="J1" s="11"/>
       <c r="M1" s="11"/>
       <c r="P1" s="11"/>
       <c r="S1" s="11"/>
     </row>
-    <row r="2" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B2" s="12"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -1232,7 +2280,7 @@
       <c r="R2" s="20"/>
       <c r="S2" s="12"/>
     </row>
-    <row r="3" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B3" s="12"/>
       <c r="C3" s="2"/>
       <c r="D3" s="57">
@@ -1274,7 +2322,7 @@
       </c>
       <c r="S3" s="12"/>
     </row>
-    <row r="4" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B4" s="33"/>
       <c r="C4" s="6" t="s">
         <v>26</v>
@@ -1296,7 +2344,7 @@
       <c r="R4" s="7"/>
       <c r="S4" s="33"/>
     </row>
-    <row r="5" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B5" s="34"/>
       <c r="C5" s="37" t="s">
         <v>1</v>
@@ -1355,7 +2403,7 @@
       <c r="AH5" s="81"/>
       <c r="AI5" s="81"/>
     </row>
-    <row r="6" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B6" s="34"/>
       <c r="C6" s="9" t="s">
         <v>12</v>
@@ -1414,7 +2462,7 @@
       <c r="AH6" s="81"/>
       <c r="AI6" s="81"/>
     </row>
-    <row r="7" spans="1:35" ht="26" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" ht="26.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1"/>
       <c r="B7" s="34"/>
       <c r="C7" s="9" t="s">
@@ -1474,7 +2522,7 @@
       <c r="AH7" s="81"/>
       <c r="AI7" s="81"/>
     </row>
-    <row r="8" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1"/>
       <c r="B8" s="34"/>
       <c r="C8" s="9" t="s">
@@ -1534,7 +2582,7 @@
       <c r="AH8" s="81"/>
       <c r="AI8" s="81"/>
     </row>
-    <row r="9" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B9" s="34"/>
       <c r="C9" s="39" t="s">
         <v>16</v>
@@ -1593,7 +2641,7 @@
       <c r="AH9" s="81"/>
       <c r="AI9" s="81"/>
     </row>
-    <row r="10" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1"/>
       <c r="B10" s="34"/>
       <c r="C10" s="9" t="s">
@@ -1653,7 +2701,7 @@
       <c r="AH10" s="81"/>
       <c r="AI10" s="81"/>
     </row>
-    <row r="11" spans="1:35" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" ht="30" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1"/>
       <c r="B11" s="34"/>
       <c r="C11" s="9" t="s">
@@ -1713,7 +2761,7 @@
       <c r="AH11" s="81"/>
       <c r="AI11" s="81"/>
     </row>
-    <row r="12" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1"/>
       <c r="B12" s="34"/>
       <c r="C12" s="9" t="s">
@@ -1773,7 +2821,7 @@
       <c r="AH12" s="81"/>
       <c r="AI12" s="81"/>
     </row>
-    <row r="13" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B13" s="35"/>
       <c r="C13" s="30" t="s">
         <v>2</v>
@@ -1810,7 +2858,7 @@
       <c r="AH13" s="81"/>
       <c r="AI13" s="81"/>
     </row>
-    <row r="14" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B14" s="34"/>
       <c r="C14" s="37" t="s">
         <v>1</v>
@@ -1869,7 +2917,7 @@
       <c r="AH14" s="81"/>
       <c r="AI14" s="81"/>
     </row>
-    <row r="15" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B15" s="34"/>
       <c r="C15" s="9" t="s">
         <v>12</v>
@@ -1928,7 +2976,7 @@
       <c r="AH15" s="81"/>
       <c r="AI15" s="81"/>
     </row>
-    <row r="16" spans="1:35" ht="32.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1"/>
       <c r="B16" s="34"/>
       <c r="C16" s="9" t="s">
@@ -1988,7 +3036,7 @@
       <c r="AH16" s="81"/>
       <c r="AI16" s="81"/>
     </row>
-    <row r="17" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1"/>
       <c r="B17" s="34"/>
       <c r="C17" s="9" t="s">
@@ -2048,7 +3096,7 @@
       <c r="AH17" s="81"/>
       <c r="AI17" s="81"/>
     </row>
-    <row r="18" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B18" s="35"/>
       <c r="C18" s="30" t="s">
         <v>19</v>
@@ -2085,7 +3133,7 @@
       <c r="AH18" s="81"/>
       <c r="AI18" s="81"/>
     </row>
-    <row r="19" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B19" s="34"/>
       <c r="C19" s="37" t="s">
         <v>1</v>
@@ -2144,7 +3192,7 @@
       <c r="AH19" s="81"/>
       <c r="AI19" s="81"/>
     </row>
-    <row r="20" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B20" s="34"/>
       <c r="C20" s="9" t="s">
         <v>12</v>
@@ -2203,7 +3251,7 @@
       <c r="AH20" s="81"/>
       <c r="AI20" s="81"/>
     </row>
-    <row r="21" spans="1:35" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:35" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1"/>
       <c r="B21" s="34"/>
       <c r="C21" s="9" t="s">
@@ -2263,7 +3311,7 @@
       <c r="AH21" s="81"/>
       <c r="AI21" s="81"/>
     </row>
-    <row r="22" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="1"/>
       <c r="B22" s="34"/>
       <c r="C22" s="9" t="s">
@@ -2323,7 +3371,7 @@
       <c r="AH22" s="81"/>
       <c r="AI22" s="81"/>
     </row>
-    <row r="23" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B23" s="35"/>
       <c r="C23" s="30" t="s">
         <v>27</v>
@@ -2360,7 +3408,7 @@
       <c r="AH23" s="81"/>
       <c r="AI23" s="81"/>
     </row>
-    <row r="24" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B24" s="34"/>
       <c r="C24" s="37" t="s">
         <v>1</v>
@@ -2419,7 +3467,7 @@
       <c r="AH24" s="81"/>
       <c r="AI24" s="81"/>
     </row>
-    <row r="25" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" s="34"/>
       <c r="C25" s="9" t="s">
         <v>12</v>
@@ -2478,7 +3526,7 @@
       <c r="AH25" s="81"/>
       <c r="AI25" s="81"/>
     </row>
-    <row r="26" spans="1:35" ht="26.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:35" ht="26.45" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="1"/>
       <c r="B26" s="34"/>
       <c r="C26" s="9" t="s">
@@ -2538,7 +3586,7 @@
       <c r="AH26" s="81"/>
       <c r="AI26" s="81"/>
     </row>
-    <row r="27" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="1"/>
       <c r="B27" s="34"/>
       <c r="C27" s="9" t="s">
@@ -2598,7 +3646,7 @@
       <c r="AH27" s="81"/>
       <c r="AI27" s="81"/>
     </row>
-    <row r="28" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1"/>
       <c r="B28" s="34"/>
       <c r="C28" s="39" t="s">
@@ -2658,7 +3706,7 @@
       <c r="AH28" s="81"/>
       <c r="AI28" s="81"/>
     </row>
-    <row r="29" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1"/>
       <c r="B29" s="34"/>
       <c r="C29" s="9" t="s">
@@ -2718,7 +3766,7 @@
       <c r="AH29" s="81"/>
       <c r="AI29" s="81"/>
     </row>
-    <row r="30" spans="1:35" ht="23" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:35" ht="23.1" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1"/>
       <c r="B30" s="34"/>
       <c r="C30" s="9" t="s">
@@ -2778,7 +3826,7 @@
       <c r="AH30" s="81"/>
       <c r="AI30" s="81"/>
     </row>
-    <row r="31" spans="1:35" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:35" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="36"/>
       <c r="C31" s="26" t="s">
@@ -2838,7 +3886,7 @@
       <c r="AH31" s="81"/>
       <c r="AI31" s="81"/>
     </row>
-    <row r="32" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C32" s="17" t="s">
         <v>17</v>
       </c>
@@ -2860,7 +3908,7 @@
       <c r="S32" s="17"/>
       <c r="T32" s="17"/>
     </row>
-    <row r="33" spans="3:19" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:19" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C33" s="17"/>
       <c r="D33" s="17"/>
       <c r="E33" s="17"/>
@@ -2879,28 +3927,28 @@
       <c r="R33" s="17"/>
       <c r="S33" s="14"/>
     </row>
-    <row r="34" spans="3:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:19" x14ac:dyDescent="0.15">
       <c r="G34" s="14"/>
       <c r="J34" s="14"/>
       <c r="M34" s="14"/>
       <c r="P34" s="14"/>
       <c r="S34" s="14"/>
     </row>
-    <row r="35" spans="3:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:19" x14ac:dyDescent="0.15">
       <c r="G35" s="13"/>
       <c r="J35" s="13"/>
       <c r="M35" s="13"/>
       <c r="P35" s="13"/>
       <c r="S35" s="13"/>
     </row>
-    <row r="36" spans="3:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:19" x14ac:dyDescent="0.15">
       <c r="G36" s="15"/>
       <c r="J36" s="15"/>
       <c r="M36" s="15"/>
       <c r="P36" s="15"/>
       <c r="S36" s="15"/>
     </row>
-    <row r="37" spans="3:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:19" x14ac:dyDescent="0.15">
       <c r="G37" s="16"/>
       <c r="J37" s="16"/>
       <c r="M37" s="16"/>
@@ -2920,17 +3968,18 @@
     <tabColor theme="8" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="B1:N75"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="2" max="2" width="31.81640625" customWidth="1"/>
-    <col min="3" max="5" width="14.26953125" customWidth="1"/>
-    <col min="6" max="6" width="0.26953125" style="18" customWidth="1"/>
-    <col min="7" max="7" width="14.26953125" customWidth="1"/>
-    <col min="8" max="8" width="0.26953125" style="18" customWidth="1"/>
-    <col min="9" max="9" width="14.7265625" customWidth="1"/>
+    <col min="2" max="2" width="31.875" customWidth="1"/>
+    <col min="3" max="5" width="14.25" customWidth="1"/>
+    <col min="6" max="6" width="0.25" style="18" customWidth="1"/>
+    <col min="7" max="7" width="14.25" customWidth="1"/>
+    <col min="8" max="8" width="0.25" style="18" customWidth="1"/>
+    <col min="9" max="9" width="14.75" customWidth="1"/>
+    <col min="10" max="10" width="12.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B1" s="9"/>
       <c r="C1" s="10"/>
       <c r="D1" s="10"/>
@@ -2939,7 +3988,7 @@
       <c r="G1" s="10"/>
       <c r="H1" s="34"/>
     </row>
-    <row r="2" spans="2:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B2" s="23" t="s">
         <v>18</v>
       </c>
@@ -2950,7 +3999,7 @@
       <c r="G2" s="24"/>
       <c r="H2" s="34"/>
     </row>
-    <row r="3" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="65"/>
@@ -2961,7 +4010,7 @@
       </c>
       <c r="H3" s="12"/>
     </row>
-    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B4" s="2"/>
       <c r="C4" s="2">
         <v>2020</v>
@@ -2978,7 +4027,7 @@
       </c>
       <c r="H4" s="12"/>
     </row>
-    <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B5" s="59" t="s">
         <v>31</v>
       </c>
@@ -2989,7 +4038,7 @@
       <c r="G5" s="7"/>
       <c r="H5" s="33"/>
     </row>
-    <row r="6" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B6" s="60" t="s">
         <v>0</v>
       </c>
@@ -3015,7 +4064,7 @@
       <c r="M6" s="79"/>
       <c r="N6" s="79"/>
     </row>
-    <row r="7" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B7" s="60" t="s">
         <v>3</v>
       </c>
@@ -3041,7 +4090,7 @@
       <c r="M7" s="79"/>
       <c r="N7" s="79"/>
     </row>
-    <row r="8" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B8" s="61" t="s">
         <v>4</v>
       </c>
@@ -3067,7 +4116,7 @@
       <c r="M8" s="79"/>
       <c r="N8" s="79"/>
     </row>
-    <row r="9" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B9" s="60" t="s">
         <v>5</v>
       </c>
@@ -3093,7 +4142,7 @@
       <c r="M9" s="79"/>
       <c r="N9" s="80"/>
     </row>
-    <row r="10" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B10" s="60" t="s">
         <v>6</v>
       </c>
@@ -3119,7 +4168,7 @@
       <c r="M10" s="79"/>
       <c r="N10" s="79"/>
     </row>
-    <row r="11" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="60" t="s">
         <v>7</v>
       </c>
@@ -3145,7 +4194,7 @@
       <c r="M11" s="79"/>
       <c r="N11" s="80"/>
     </row>
-    <row r="12" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B12" s="60" t="s">
         <v>8</v>
       </c>
@@ -3171,7 +4220,7 @@
       <c r="M12" s="79"/>
       <c r="N12" s="80"/>
     </row>
-    <row r="13" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B13" s="60" t="s">
         <v>9</v>
       </c>
@@ -3197,7 +4246,7 @@
       <c r="M13" s="79"/>
       <c r="N13" s="79"/>
     </row>
-    <row r="14" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B14" s="61" t="s">
         <v>10</v>
       </c>
@@ -3223,7 +4272,7 @@
       <c r="M14" s="79"/>
       <c r="N14" s="79"/>
     </row>
-    <row r="15" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B15" s="63" t="s">
         <v>32</v>
       </c>
@@ -3239,7 +4288,7 @@
       <c r="M15" s="79"/>
       <c r="N15" s="79"/>
     </row>
-    <row r="16" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B16" s="60" t="s">
         <v>0</v>
       </c>
@@ -3265,7 +4314,7 @@
       <c r="M16" s="79"/>
       <c r="N16" s="79"/>
     </row>
-    <row r="17" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B17" s="60" t="s">
         <v>3</v>
       </c>
@@ -3291,7 +4340,7 @@
       <c r="M17" s="79"/>
       <c r="N17" s="79"/>
     </row>
-    <row r="18" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B18" s="61" t="s">
         <v>4</v>
       </c>
@@ -3317,7 +4366,7 @@
       <c r="M18" s="79"/>
       <c r="N18" s="79"/>
     </row>
-    <row r="19" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B19" s="60" t="s">
         <v>5</v>
       </c>
@@ -3343,7 +4392,7 @@
       <c r="M19" s="79"/>
       <c r="N19" s="80"/>
     </row>
-    <row r="20" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B20" s="60" t="s">
         <v>6</v>
       </c>
@@ -3369,7 +4418,7 @@
       <c r="M20" s="79"/>
       <c r="N20" s="79"/>
     </row>
-    <row r="21" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B21" s="60" t="s">
         <v>7</v>
       </c>
@@ -3395,7 +4444,7 @@
       <c r="M21" s="79"/>
       <c r="N21" s="80"/>
     </row>
-    <row r="22" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B22" s="60" t="s">
         <v>8</v>
       </c>
@@ -3421,7 +4470,7 @@
       <c r="M22" s="79"/>
       <c r="N22" s="80"/>
     </row>
-    <row r="23" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B23" s="60" t="s">
         <v>9</v>
       </c>
@@ -3447,7 +4496,7 @@
       <c r="M23" s="79"/>
       <c r="N23" s="79"/>
     </row>
-    <row r="24" spans="2:14" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:14" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B24" s="62" t="s">
         <v>10</v>
       </c>
@@ -3473,7 +4522,7 @@
       <c r="M24" s="79"/>
       <c r="N24" s="79"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B25" s="9"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
@@ -3482,7 +4531,7 @@
       <c r="G25" s="75"/>
       <c r="H25" s="34"/>
     </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B26" s="9"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
@@ -3491,7 +4540,7 @@
       <c r="G26" s="10"/>
       <c r="H26" s="34"/>
     </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B27" s="23" t="s">
         <v>21</v>
       </c>
@@ -3502,7 +4551,7 @@
       <c r="G27" s="24"/>
       <c r="H27" s="34"/>
     </row>
-    <row r="28" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -3513,7 +4562,7 @@
       </c>
       <c r="H28" s="12"/>
     </row>
-    <row r="29" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B29" s="2"/>
       <c r="C29" s="2">
         <v>2020</v>
@@ -3530,7 +4579,7 @@
       </c>
       <c r="H29" s="12"/>
     </row>
-    <row r="30" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B30" s="59" t="s">
         <v>2</v>
       </c>
@@ -3541,7 +4590,7 @@
       <c r="G30" s="7"/>
       <c r="H30" s="33"/>
     </row>
-    <row r="31" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B31" s="60" t="s">
         <v>0</v>
       </c>
@@ -3561,13 +4610,16 @@
         <v>1.29</v>
       </c>
       <c r="H31" s="34"/>
-      <c r="J31" s="79"/>
+      <c r="J31" s="107">
+        <f>E6/E16</f>
+        <v>1.4264705882352942</v>
+      </c>
       <c r="K31" s="79"/>
       <c r="L31" s="79"/>
       <c r="M31" s="79"/>
       <c r="N31" s="79"/>
     </row>
-    <row r="32" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B32" s="60" t="s">
         <v>3</v>
       </c>
@@ -3587,13 +4639,16 @@
         <v>1.24</v>
       </c>
       <c r="H32" s="34"/>
-      <c r="J32" s="79"/>
+      <c r="J32" s="107">
+        <f t="shared" ref="J32:J39" si="0">E7/E17</f>
+        <v>1.34375</v>
+      </c>
       <c r="K32" s="79"/>
       <c r="L32" s="79"/>
       <c r="M32" s="79"/>
       <c r="N32" s="79"/>
     </row>
-    <row r="33" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B33" s="61" t="s">
         <v>4</v>
       </c>
@@ -3613,13 +4668,16 @@
         <v>1.23</v>
       </c>
       <c r="H33" s="34"/>
-      <c r="J33" s="79"/>
+      <c r="J33" s="107">
+        <f t="shared" si="0"/>
+        <v>1.3548387096774193</v>
+      </c>
       <c r="K33" s="79"/>
       <c r="L33" s="79"/>
       <c r="M33" s="79"/>
       <c r="N33" s="79"/>
     </row>
-    <row r="34" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B34" s="60" t="s">
         <v>5</v>
       </c>
@@ -3639,13 +4697,16 @@
         <v>1.5</v>
       </c>
       <c r="H34" s="34"/>
-      <c r="J34" s="79"/>
+      <c r="J34" s="107">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
       <c r="K34" s="79"/>
       <c r="L34" s="79"/>
       <c r="M34" s="79"/>
       <c r="N34" s="79"/>
     </row>
-    <row r="35" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B35" s="60" t="s">
         <v>6</v>
       </c>
@@ -3665,13 +4726,16 @@
         <v>1.29</v>
       </c>
       <c r="H35" s="34"/>
-      <c r="J35" s="79"/>
+      <c r="J35" s="107">
+        <f t="shared" si="0"/>
+        <v>1.4545454545454546</v>
+      </c>
       <c r="K35" s="79"/>
       <c r="L35" s="79"/>
       <c r="M35" s="79"/>
       <c r="N35" s="79"/>
     </row>
-    <row r="36" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B36" s="60" t="s">
         <v>7</v>
       </c>
@@ -3691,13 +4755,16 @@
         <v>1.59</v>
       </c>
       <c r="H36" s="34"/>
-      <c r="J36" s="79"/>
+      <c r="J36" s="107">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
       <c r="K36" s="79"/>
       <c r="L36" s="79"/>
       <c r="M36" s="79"/>
       <c r="N36" s="79"/>
     </row>
-    <row r="37" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B37" s="60" t="s">
         <v>8</v>
       </c>
@@ -3717,13 +4784,16 @@
         <v>1.7</v>
       </c>
       <c r="H37" s="34"/>
-      <c r="J37" s="79"/>
+      <c r="J37" s="107">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
       <c r="K37" s="79"/>
       <c r="L37" s="79"/>
       <c r="M37" s="79"/>
       <c r="N37" s="79"/>
     </row>
-    <row r="38" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B38" s="60" t="s">
         <v>9</v>
       </c>
@@ -3743,13 +4813,16 @@
         <v>1.35</v>
       </c>
       <c r="H38" s="34"/>
-      <c r="J38" s="79"/>
+      <c r="J38" s="107">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
       <c r="K38" s="79"/>
       <c r="L38" s="79"/>
       <c r="M38" s="79"/>
       <c r="N38" s="79"/>
     </row>
-    <row r="39" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B39" s="61" t="s">
         <v>10</v>
       </c>
@@ -3769,13 +4842,16 @@
         <v>1.35</v>
       </c>
       <c r="H39" s="34"/>
-      <c r="J39" s="79"/>
+      <c r="J39" s="107">
+        <f t="shared" si="0"/>
+        <v>1.5</v>
+      </c>
       <c r="K39" s="79"/>
       <c r="L39" s="79"/>
       <c r="M39" s="79"/>
       <c r="N39" s="79"/>
     </row>
-    <row r="40" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B40" s="63" t="s">
         <v>30</v>
       </c>
@@ -3791,7 +4867,7 @@
       <c r="M40" s="79"/>
       <c r="N40" s="79"/>
     </row>
-    <row r="41" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B41" s="60" t="s">
         <v>0</v>
       </c>
@@ -3811,13 +4887,16 @@
         <v>48</v>
       </c>
       <c r="H41" s="34"/>
-      <c r="J41" s="79"/>
+      <c r="J41" s="106">
+        <f>E6*E41/10</f>
+        <v>475.3</v>
+      </c>
       <c r="K41" s="79"/>
       <c r="L41" s="79"/>
       <c r="M41" s="79"/>
       <c r="N41" s="79"/>
     </row>
-    <row r="42" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B42" s="60" t="s">
         <v>3</v>
       </c>
@@ -3837,13 +4916,16 @@
         <v>48</v>
       </c>
       <c r="H42" s="34"/>
-      <c r="J42" s="79"/>
+      <c r="J42" s="106">
+        <f t="shared" ref="J42:J49" si="1">E7*E42/10</f>
+        <v>215</v>
+      </c>
       <c r="K42" s="79"/>
       <c r="L42" s="79"/>
       <c r="M42" s="79"/>
       <c r="N42" s="79"/>
     </row>
-    <row r="43" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B43" s="61" t="s">
         <v>4</v>
       </c>
@@ -3863,13 +4945,16 @@
         <v>49</v>
       </c>
       <c r="H43" s="34"/>
-      <c r="J43" s="79"/>
+      <c r="J43" s="106">
+        <f t="shared" si="1"/>
+        <v>210</v>
+      </c>
       <c r="K43" s="79"/>
       <c r="L43" s="79"/>
       <c r="M43" s="79"/>
       <c r="N43" s="79"/>
     </row>
-    <row r="44" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B44" s="60" t="s">
         <v>5</v>
       </c>
@@ -3889,13 +4974,16 @@
         <v>46</v>
       </c>
       <c r="H44" s="34"/>
-      <c r="J44" s="79"/>
+      <c r="J44" s="106">
+        <f t="shared" si="1"/>
+        <v>1.8800000000000001</v>
+      </c>
       <c r="K44" s="79"/>
       <c r="L44" s="79"/>
       <c r="M44" s="79"/>
       <c r="N44" s="79"/>
     </row>
-    <row r="45" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B45" s="60" t="s">
         <v>6</v>
       </c>
@@ -3915,13 +5003,16 @@
         <v>48</v>
       </c>
       <c r="H45" s="34"/>
-      <c r="J45" s="79"/>
+      <c r="J45" s="106">
+        <f t="shared" si="1"/>
+        <v>76.8</v>
+      </c>
       <c r="K45" s="79"/>
       <c r="L45" s="79"/>
       <c r="M45" s="79"/>
       <c r="N45" s="79"/>
     </row>
-    <row r="46" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B46" s="60" t="s">
         <v>7</v>
       </c>
@@ -3941,13 +5032,16 @@
         <v>45</v>
       </c>
       <c r="H46" s="34"/>
-      <c r="J46" s="79"/>
+      <c r="J46" s="106">
+        <f t="shared" si="1"/>
+        <v>1.8400000000000003</v>
+      </c>
       <c r="K46" s="79"/>
       <c r="L46" s="79"/>
       <c r="M46" s="79"/>
       <c r="N46" s="79"/>
     </row>
-    <row r="47" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B47" s="60" t="s">
         <v>8</v>
       </c>
@@ -3967,13 +5061,16 @@
         <v>45</v>
       </c>
       <c r="H47" s="34"/>
-      <c r="J47" s="79"/>
+      <c r="J47" s="106">
+        <f t="shared" si="1"/>
+        <v>1.8400000000000003</v>
+      </c>
       <c r="K47" s="79"/>
       <c r="L47" s="79"/>
       <c r="M47" s="79"/>
       <c r="N47" s="79"/>
     </row>
-    <row r="48" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B48" s="60" t="s">
         <v>9</v>
       </c>
@@ -3993,13 +5090,16 @@
         <v>47</v>
       </c>
       <c r="H48" s="34"/>
-      <c r="J48" s="79"/>
+      <c r="J48" s="106">
+        <f t="shared" si="1"/>
+        <v>172.8</v>
+      </c>
       <c r="K48" s="79"/>
       <c r="L48" s="79"/>
       <c r="M48" s="79"/>
       <c r="N48" s="79"/>
     </row>
-    <row r="49" spans="2:14" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:14" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B49" s="62" t="s">
         <v>10</v>
       </c>
@@ -4019,13 +5119,16 @@
         <v>47</v>
       </c>
       <c r="H49" s="71"/>
-      <c r="J49" s="79"/>
+      <c r="J49" s="106">
+        <f t="shared" si="1"/>
+        <v>115.2</v>
+      </c>
       <c r="K49" s="79"/>
       <c r="L49" s="79"/>
       <c r="M49" s="79"/>
       <c r="N49" s="79"/>
     </row>
-    <row r="50" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B50" s="9"/>
       <c r="C50" s="5"/>
       <c r="D50" s="5"/>
@@ -4034,7 +5137,7 @@
       <c r="G50" s="77"/>
       <c r="H50" s="34"/>
     </row>
-    <row r="51" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B51" s="9"/>
       <c r="C51" s="5"/>
       <c r="D51" s="5"/>
@@ -4043,7 +5146,7 @@
       <c r="G51" s="5"/>
       <c r="H51" s="34"/>
     </row>
-    <row r="52" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B52" s="9"/>
       <c r="C52" s="5"/>
       <c r="D52" s="5"/>
@@ -4052,7 +5155,7 @@
       <c r="G52" s="5"/>
       <c r="H52" s="34"/>
     </row>
-    <row r="53" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:14" x14ac:dyDescent="0.15">
       <c r="B53" s="23" t="s">
         <v>20</v>
       </c>
@@ -4063,7 +5166,7 @@
       <c r="G53" s="24"/>
       <c r="H53" s="34"/>
     </row>
-    <row r="54" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
@@ -4074,7 +5177,7 @@
       </c>
       <c r="H54" s="12"/>
     </row>
-    <row r="55" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B55" s="2"/>
       <c r="C55" s="2">
         <v>2020</v>
@@ -4091,7 +5194,7 @@
       </c>
       <c r="H55" s="12"/>
     </row>
-    <row r="56" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B56" s="59" t="s">
         <v>28</v>
       </c>
@@ -4102,7 +5205,7 @@
       <c r="G56" s="7"/>
       <c r="H56" s="33"/>
     </row>
-    <row r="57" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B57" s="60" t="s">
         <v>0</v>
       </c>
@@ -4128,7 +5231,7 @@
       <c r="M57" s="79"/>
       <c r="N57" s="79"/>
     </row>
-    <row r="58" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B58" s="60" t="s">
         <v>3</v>
       </c>
@@ -4154,7 +5257,7 @@
       <c r="M58" s="79"/>
       <c r="N58" s="79"/>
     </row>
-    <row r="59" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B59" s="61" t="s">
         <v>4</v>
       </c>
@@ -4180,7 +5283,7 @@
       <c r="M59" s="79"/>
       <c r="N59" s="79"/>
     </row>
-    <row r="60" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B60" s="60" t="s">
         <v>5</v>
       </c>
@@ -4207,7 +5310,7 @@
       <c r="M60" s="79"/>
       <c r="N60" s="80"/>
     </row>
-    <row r="61" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B61" s="60" t="s">
         <v>6</v>
       </c>
@@ -4234,7 +5337,7 @@
       <c r="M61" s="79"/>
       <c r="N61" s="79"/>
     </row>
-    <row r="62" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B62" s="60" t="s">
         <v>7</v>
       </c>
@@ -4261,7 +5364,7 @@
       <c r="M62" s="79"/>
       <c r="N62" s="80"/>
     </row>
-    <row r="63" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B63" s="60" t="s">
         <v>8</v>
       </c>
@@ -4288,7 +5391,7 @@
       <c r="M63" s="79"/>
       <c r="N63" s="80"/>
     </row>
-    <row r="64" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B64" s="60" t="s">
         <v>9</v>
       </c>
@@ -4315,7 +5418,7 @@
       <c r="M64" s="79"/>
       <c r="N64" s="79"/>
     </row>
-    <row r="65" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B65" s="61" t="s">
         <v>10</v>
       </c>
@@ -4342,7 +5445,7 @@
       <c r="M65" s="79"/>
       <c r="N65" s="79"/>
     </row>
-    <row r="66" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B66" s="63" t="s">
         <v>29</v>
       </c>
@@ -4358,7 +5461,7 @@
       <c r="M66" s="79"/>
       <c r="N66" s="79"/>
     </row>
-    <row r="67" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B67" s="60" t="s">
         <v>0</v>
       </c>
@@ -4384,7 +5487,7 @@
       <c r="M67" s="79"/>
       <c r="N67" s="79"/>
     </row>
-    <row r="68" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B68" s="60" t="s">
         <v>3</v>
       </c>
@@ -4410,7 +5513,7 @@
       <c r="M68" s="79"/>
       <c r="N68" s="79"/>
     </row>
-    <row r="69" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B69" s="61" t="s">
         <v>4</v>
       </c>
@@ -4436,7 +5539,7 @@
       <c r="M69" s="79"/>
       <c r="N69" s="79"/>
     </row>
-    <row r="70" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B70" s="60" t="s">
         <v>5</v>
       </c>
@@ -4462,7 +5565,7 @@
       <c r="M70" s="79"/>
       <c r="N70" s="80"/>
     </row>
-    <row r="71" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B71" s="60" t="s">
         <v>6</v>
       </c>
@@ -4488,7 +5591,7 @@
       <c r="M71" s="79"/>
       <c r="N71" s="79"/>
     </row>
-    <row r="72" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B72" s="60" t="s">
         <v>7</v>
       </c>
@@ -4514,7 +5617,7 @@
       <c r="M72" s="79"/>
       <c r="N72" s="80"/>
     </row>
-    <row r="73" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B73" s="60" t="s">
         <v>8</v>
       </c>
@@ -4540,7 +5643,7 @@
       <c r="M73" s="79"/>
       <c r="N73" s="80"/>
     </row>
-    <row r="74" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B74" s="60" t="s">
         <v>9</v>
       </c>
@@ -4566,7 +5669,7 @@
       <c r="M74" s="79"/>
       <c r="N74" s="79"/>
     </row>
-    <row r="75" spans="2:14" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="2:14" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="B75" s="62" t="s">
         <v>10</v>
       </c>
@@ -4596,5 +5699,6 @@
   <phoneticPr fontId="15" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>